<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@49cbe7ccf48a3eb74bcd203e5cc07992300ad171 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-DocumentReference.xlsx
+++ b/StructureDefinition-DocumentReference.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$66</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2273" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2417" uniqueCount="475">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-05-03T08:33:55+00:00</t>
+    <t>2024-05-07T11:45:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1304,6 +1304,61 @@
   </si>
   <si>
     <t>DocumentEntry.serviceStartTime DocumentEntry.serviceStopTime</t>
+  </si>
+  <si>
+    <t>DocumentReference.context.period.id</t>
+  </si>
+  <si>
+    <t>DocumentReference.context.period.extension</t>
+  </si>
+  <si>
+    <t>DocumentReference.context.period.start</t>
+  </si>
+  <si>
+    <t>Starting time with inclusive boundary</t>
+  </si>
+  <si>
+    <t>The start of the period. The boundary is inclusive.</t>
+  </si>
+  <si>
+    <t>If the low element is missing, the meaning is that the low boundary is not known.</t>
+  </si>
+  <si>
+    <t>Period.start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">per-1
+</t>
+  </si>
+  <si>
+    <t>./low</t>
+  </si>
+  <si>
+    <t>DR.1</t>
+  </si>
+  <si>
+    <t>DocumentReference.context.period.end</t>
+  </si>
+  <si>
+    <t>End time with inclusive boundary, if not ongoing</t>
+  </si>
+  <si>
+    <t>The end of the period. If the end of the period is missing, it means that the period is ongoing. The start may be in the past, and the end date in the future, which means that period is expected/planned to end at that time.</t>
+  </si>
+  <si>
+    <t>The high value includes any matching date/time. i.e. 2012-02-03T10:00:00 is in a period that has a end value of 2012-02-03.</t>
+  </si>
+  <si>
+    <t>If the end of the period is missing, it means that the period is ongoing</t>
+  </si>
+  <si>
+    <t>Period.end</t>
+  </si>
+  <si>
+    <t>./high</t>
+  </si>
+  <si>
+    <t>DR.2</t>
   </si>
   <si>
     <t>DocumentReference.context.facilityType</t>
@@ -1750,7 +1805,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN62"/>
+  <dimension ref="A1:AN66"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="51.73046875" customWidth="true" bestFit="true"/>
@@ -7861,22 +7916,22 @@
         <v>87</v>
       </c>
       <c r="H54" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="I54" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J54" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>179</v>
+        <v>257</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>418</v>
+        <v>258</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>419</v>
+        <v>259</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -7903,13 +7958,13 @@
         <v>76</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>196</v>
+        <v>76</v>
       </c>
       <c r="Y54" t="s" s="2">
-        <v>420</v>
+        <v>76</v>
       </c>
       <c r="Z54" t="s" s="2">
-        <v>421</v>
+        <v>76</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>76</v>
@@ -7927,7 +7982,7 @@
         <v>76</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>417</v>
+        <v>260</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>77</v>
@@ -7942,7 +7997,7 @@
         <v>76</v>
       </c>
       <c r="AK54" t="s" s="2">
-        <v>422</v>
+        <v>261</v>
       </c>
       <c r="AL54" t="s" s="2">
         <v>76</v>
@@ -7951,51 +8006,49 @@
         <v>76</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>423</v>
+        <v>76</v>
       </c>
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G55" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H55" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="I55" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J55" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>179</v>
+        <v>133</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>425</v>
+        <v>134</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>426</v>
+        <v>263</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>427</v>
-      </c>
-      <c r="O55" t="s" s="2">
-        <v>428</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
         <v>76</v>
       </c>
@@ -8019,37 +8072,37 @@
         <v>76</v>
       </c>
       <c r="X55" t="s" s="2">
-        <v>196</v>
+        <v>76</v>
       </c>
       <c r="Y55" t="s" s="2">
-        <v>429</v>
+        <v>76</v>
       </c>
       <c r="Z55" t="s" s="2">
-        <v>430</v>
+        <v>76</v>
       </c>
       <c r="AA55" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AB55" t="s" s="2">
-        <v>76</v>
+        <v>317</v>
       </c>
       <c r="AC55" t="s" s="2">
-        <v>76</v>
+        <v>318</v>
       </c>
       <c r="AD55" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE55" t="s" s="2">
-        <v>76</v>
+        <v>319</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>424</v>
+        <v>264</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH55" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI55" t="s" s="2">
         <v>76</v>
@@ -8058,7 +8111,7 @@
         <v>76</v>
       </c>
       <c r="AK55" t="s" s="2">
-        <v>422</v>
+        <v>261</v>
       </c>
       <c r="AL55" t="s" s="2">
         <v>76</v>
@@ -8067,15 +8120,15 @@
         <v>76</v>
       </c>
       <c r="AN55" t="s" s="2">
-        <v>431</v>
+        <v>76</v>
       </c>
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>432</v>
+        <v>419</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>432</v>
+        <v>419</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8098,16 +8151,16 @@
         <v>88</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>236</v>
+        <v>211</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>433</v>
+        <v>420</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>434</v>
+        <v>421</v>
       </c>
       <c r="N56" t="s" s="2">
-        <v>435</v>
+        <v>422</v>
       </c>
       <c r="O56" s="2"/>
       <c r="P56" t="s" s="2">
@@ -8157,7 +8210,7 @@
         <v>76</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>432</v>
+        <v>423</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>77</v>
@@ -8166,30 +8219,30 @@
         <v>87</v>
       </c>
       <c r="AI56" t="s" s="2">
-        <v>76</v>
+        <v>424</v>
       </c>
       <c r="AJ56" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AK56" t="s" s="2">
-        <v>206</v>
+        <v>425</v>
       </c>
       <c r="AL56" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AM56" t="s" s="2">
-        <v>76</v>
+        <v>426</v>
       </c>
       <c r="AN56" t="s" s="2">
-        <v>436</v>
+        <v>76</v>
       </c>
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>437</v>
+        <v>427</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>437</v>
+        <v>427</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8200,7 +8253,7 @@
         <v>77</v>
       </c>
       <c r="G57" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H57" t="s" s="2">
         <v>76</v>
@@ -8212,22 +8265,24 @@
         <v>88</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>250</v>
+        <v>211</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>438</v>
+        <v>428</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>439</v>
+        <v>429</v>
       </c>
       <c r="N57" t="s" s="2">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
         <v>76</v>
       </c>
-      <c r="Q57" s="2"/>
+      <c r="Q57" t="s" s="2">
+        <v>431</v>
+      </c>
       <c r="R57" t="s" s="2">
         <v>76</v>
       </c>
@@ -8271,39 +8326,39 @@
         <v>76</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH57" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI57" t="s" s="2">
-        <v>76</v>
+        <v>424</v>
       </c>
       <c r="AJ57" t="s" s="2">
-        <v>254</v>
+        <v>76</v>
       </c>
       <c r="AK57" t="s" s="2">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="AL57" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AM57" t="s" s="2">
-        <v>76</v>
+        <v>434</v>
       </c>
       <c r="AN57" t="s" s="2">
-        <v>442</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8317,22 +8372,22 @@
         <v>87</v>
       </c>
       <c r="H58" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="I58" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J58" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>257</v>
+        <v>179</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>258</v>
+        <v>436</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>259</v>
+        <v>437</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -8359,13 +8414,13 @@
         <v>76</v>
       </c>
       <c r="X58" t="s" s="2">
-        <v>76</v>
+        <v>196</v>
       </c>
       <c r="Y58" t="s" s="2">
-        <v>76</v>
+        <v>438</v>
       </c>
       <c r="Z58" t="s" s="2">
-        <v>76</v>
+        <v>439</v>
       </c>
       <c r="AA58" t="s" s="2">
         <v>76</v>
@@ -8383,7 +8438,7 @@
         <v>76</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>260</v>
+        <v>435</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>77</v>
@@ -8398,7 +8453,7 @@
         <v>76</v>
       </c>
       <c r="AK58" t="s" s="2">
-        <v>261</v>
+        <v>440</v>
       </c>
       <c r="AL58" t="s" s="2">
         <v>76</v>
@@ -8407,49 +8462,51 @@
         <v>76</v>
       </c>
       <c r="AN58" t="s" s="2">
-        <v>76</v>
+        <v>441</v>
       </c>
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="E59" s="2"/>
       <c r="F59" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G59" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H59" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="I59" t="s" s="2">
         <v>76</v>
       </c>
       <c r="J59" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>133</v>
+        <v>179</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>134</v>
+        <v>443</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>263</v>
+        <v>444</v>
       </c>
       <c r="N59" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="O59" s="2"/>
+        <v>445</v>
+      </c>
+      <c r="O59" t="s" s="2">
+        <v>446</v>
+      </c>
       <c r="P59" t="s" s="2">
         <v>76</v>
       </c>
@@ -8473,13 +8530,13 @@
         <v>76</v>
       </c>
       <c r="X59" t="s" s="2">
-        <v>76</v>
+        <v>196</v>
       </c>
       <c r="Y59" t="s" s="2">
-        <v>76</v>
+        <v>447</v>
       </c>
       <c r="Z59" t="s" s="2">
-        <v>76</v>
+        <v>448</v>
       </c>
       <c r="AA59" t="s" s="2">
         <v>76</v>
@@ -8497,13 +8554,13 @@
         <v>76</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>264</v>
+        <v>442</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH59" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI59" t="s" s="2">
         <v>76</v>
@@ -8512,7 +8569,7 @@
         <v>76</v>
       </c>
       <c r="AK59" t="s" s="2">
-        <v>261</v>
+        <v>440</v>
       </c>
       <c r="AL59" t="s" s="2">
         <v>76</v>
@@ -8521,47 +8578,47 @@
         <v>76</v>
       </c>
       <c r="AN59" t="s" s="2">
-        <v>76</v>
+        <v>449</v>
       </c>
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
-        <v>266</v>
+        <v>76</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G60" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="H60" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="I60" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="J60" t="s" s="2">
         <v>88</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>133</v>
+        <v>236</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>139</v>
+        <v>451</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>267</v>
+        <v>452</v>
       </c>
       <c r="N60" t="s" s="2">
-        <v>136</v>
+        <v>453</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
@@ -8611,13 +8668,13 @@
         <v>76</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>268</v>
+        <v>450</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH60" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AI60" t="s" s="2">
         <v>76</v>
@@ -8626,7 +8683,7 @@
         <v>76</v>
       </c>
       <c r="AK60" t="s" s="2">
-        <v>130</v>
+        <v>206</v>
       </c>
       <c r="AL60" t="s" s="2">
         <v>76</v>
@@ -8635,15 +8692,15 @@
         <v>76</v>
       </c>
       <c r="AN60" t="s" s="2">
-        <v>76</v>
+        <v>454</v>
       </c>
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>446</v>
+        <v>455</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>446</v>
+        <v>455</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -8654,7 +8711,7 @@
         <v>77</v>
       </c>
       <c r="G61" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="H61" t="s" s="2">
         <v>76</v>
@@ -8666,16 +8723,16 @@
         <v>88</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>143</v>
+        <v>250</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>447</v>
+        <v>456</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>448</v>
+        <v>457</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>449</v>
+        <v>458</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -8725,22 +8782,22 @@
         <v>76</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>446</v>
+        <v>455</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH61" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AI61" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ61" t="s" s="2">
-        <v>76</v>
+        <v>254</v>
       </c>
       <c r="AK61" t="s" s="2">
-        <v>450</v>
+        <v>459</v>
       </c>
       <c r="AL61" t="s" s="2">
         <v>76</v>
@@ -8749,15 +8806,15 @@
         <v>76</v>
       </c>
       <c r="AN61" t="s" s="2">
-        <v>76</v>
+        <v>460</v>
       </c>
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>451</v>
+        <v>461</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>451</v>
+        <v>461</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -8777,20 +8834,18 @@
         <v>76</v>
       </c>
       <c r="J62" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>452</v>
+        <v>257</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>453</v>
+        <v>258</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>454</v>
-      </c>
-      <c r="N62" t="s" s="2">
-        <v>455</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="N62" s="2"/>
       <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
         <v>76</v>
@@ -8839,7 +8894,7 @@
         <v>76</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>451</v>
+        <v>260</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>77</v>
@@ -8854,7 +8909,7 @@
         <v>76</v>
       </c>
       <c r="AK62" t="s" s="2">
-        <v>456</v>
+        <v>261</v>
       </c>
       <c r="AL62" t="s" s="2">
         <v>76</v>
@@ -8863,11 +8918,467 @@
         <v>76</v>
       </c>
       <c r="AN62" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="63" hidden="true">
+      <c r="A63" t="s" s="2">
+        <v>462</v>
+      </c>
+      <c r="B63" t="s" s="2">
+        <v>462</v>
+      </c>
+      <c r="C63" s="2"/>
+      <c r="D63" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="E63" s="2"/>
+      <c r="F63" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G63" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K63" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="L63" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="M63" t="s" s="2">
+        <v>263</v>
+      </c>
+      <c r="N63" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="O63" s="2"/>
+      <c r="P63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q63" s="2"/>
+      <c r="R63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF63" t="s" s="2">
+        <v>264</v>
+      </c>
+      <c r="AG63" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH63" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK63" t="s" s="2">
+        <v>261</v>
+      </c>
+      <c r="AL63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AM63" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AN63" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="64" hidden="true">
+      <c r="A64" t="s" s="2">
+        <v>463</v>
+      </c>
+      <c r="B64" t="s" s="2">
+        <v>463</v>
+      </c>
+      <c r="C64" s="2"/>
+      <c r="D64" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="E64" s="2"/>
+      <c r="F64" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G64" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I64" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="J64" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K64" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="L64" t="s" s="2">
+        <v>139</v>
+      </c>
+      <c r="M64" t="s" s="2">
+        <v>267</v>
+      </c>
+      <c r="N64" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="O64" s="2"/>
+      <c r="P64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q64" s="2"/>
+      <c r="R64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF64" t="s" s="2">
+        <v>268</v>
+      </c>
+      <c r="AG64" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH64" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK64" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="AL64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AM64" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AN64" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="65" hidden="true">
+      <c r="A65" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="B65" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="C65" s="2"/>
+      <c r="D65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E65" s="2"/>
+      <c r="F65" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G65" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J65" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K65" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="L65" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="M65" t="s" s="2">
+        <v>466</v>
+      </c>
+      <c r="N65" t="s" s="2">
+        <v>467</v>
+      </c>
+      <c r="O65" s="2"/>
+      <c r="P65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q65" s="2"/>
+      <c r="R65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF65" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="AG65" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH65" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK65" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="AL65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AM65" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AN65" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="66" hidden="true">
+      <c r="A66" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="B66" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="C66" s="2"/>
+      <c r="D66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E66" s="2"/>
+      <c r="F66" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G66" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J66" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K66" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="L66" t="s" s="2">
+        <v>471</v>
+      </c>
+      <c r="M66" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="N66" t="s" s="2">
+        <v>473</v>
+      </c>
+      <c r="O66" s="2"/>
+      <c r="P66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q66" s="2"/>
+      <c r="R66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF66" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="AG66" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH66" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK66" t="s" s="2">
+        <v>474</v>
+      </c>
+      <c r="AL66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AM66" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AN66" t="s" s="2">
         <v>76</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN62">
+  <autoFilter ref="A1:AN66">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -8877,7 +9388,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI61">
+  <conditionalFormatting sqref="A2:AI65">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@ed6507d127b03fe721f2f3bda02747c1e0973e2d 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-DocumentReference.xlsx
+++ b/StructureDefinition-DocumentReference.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2417" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2415" uniqueCount="472">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-10-03T16:09:56+00:00</t>
+    <t>2024-10-03T16:43:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -584,13 +584,7 @@
     <t>Key metadata element describing the document, used in searching/filtering.</t>
   </si>
   <si>
-    <t>preferred</t>
-  </si>
-  <si>
-    <t>Precise type of clinical document.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/c80-doc-typecodes</t>
+    <t>http://hl7.nl/fhir/zorgviewer/ValueSet/DocumentLOINCCodelist</t>
   </si>
   <si>
     <t>./code</t>
@@ -624,15 +618,6 @@
     <t>Helps humans to assess whether the document is of interest when viewing a list of documents.</t>
   </si>
   <si>
-    <t>example</t>
-  </si>
-  <si>
-    <t>High-level kind of a clinical document at a macro level.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/c80-doc-classcodes</t>
-  </si>
-  <si>
     <t>.outboundRelationship[typeCode="COMP].target[classCode="LIST", moodCode="EVN"].code</t>
   </si>
   <si>
@@ -1211,6 +1196,9 @@
     <t>Note that while IHE mostly issues URNs for format types, not all documents can be identified by a URI.</t>
   </si>
   <si>
+    <t>preferred</t>
+  </si>
+  <si>
     <t>http://ihe.net/fhir/ValueSet/IHE.formatcode.vs</t>
   </si>
   <si>
@@ -1273,6 +1261,9 @@
   </si>
   <si>
     <t>An event can further specialize the act inherent in the type, such as  where it is simply "Procedure Report" and the procedure was a "colonoscopy". If one or more event codes are included, they shall not conflict with the values inherent in the class or type elements as such a conflict would create an ambiguous situation.</t>
+  </si>
+  <si>
+    <t>example</t>
   </si>
   <si>
     <t>This list of codes represents the main clinical acts being documented.</t>
@@ -1833,7 +1824,7 @@
     <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="18.859375" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="74.265625" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="51.71484375" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="58.125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="6.34765625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="22.71875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="42.03515625" customWidth="true" bestFit="true"/>
@@ -3516,13 +3507,11 @@
         <v>76</v>
       </c>
       <c r="X15" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="Y15" s="2"/>
+      <c r="Z15" t="s" s="2">
         <v>183</v>
-      </c>
-      <c r="Y15" t="s" s="2">
-        <v>184</v>
-      </c>
-      <c r="Z15" t="s" s="2">
-        <v>185</v>
       </c>
       <c r="AA15" t="s" s="2">
         <v>76</v>
@@ -3555,28 +3544,28 @@
         <v>76</v>
       </c>
       <c r="AK15" t="s" s="2">
+        <v>184</v>
+      </c>
+      <c r="AL15" t="s" s="2">
+        <v>185</v>
+      </c>
+      <c r="AM15" t="s" s="2">
         <v>186</v>
       </c>
-      <c r="AL15" t="s" s="2">
+      <c r="AN15" t="s" s="2">
         <v>187</v>
-      </c>
-      <c r="AM15" t="s" s="2">
-        <v>188</v>
-      </c>
-      <c r="AN15" t="s" s="2">
-        <v>189</v>
       </c>
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" t="s" s="2">
@@ -3598,16 +3587,16 @@
         <v>179</v>
       </c>
       <c r="L16" t="s" s="2">
+        <v>190</v>
+      </c>
+      <c r="M16" t="s" s="2">
+        <v>191</v>
+      </c>
+      <c r="N16" t="s" s="2">
         <v>192</v>
       </c>
-      <c r="M16" t="s" s="2">
+      <c r="O16" t="s" s="2">
         <v>193</v>
-      </c>
-      <c r="N16" t="s" s="2">
-        <v>194</v>
-      </c>
-      <c r="O16" t="s" s="2">
-        <v>195</v>
       </c>
       <c r="P16" t="s" s="2">
         <v>76</v>
@@ -3632,13 +3621,11 @@
         <v>76</v>
       </c>
       <c r="X16" t="s" s="2">
-        <v>196</v>
-      </c>
-      <c r="Y16" t="s" s="2">
-        <v>197</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="Y16" s="2"/>
       <c r="Z16" t="s" s="2">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="AA16" t="s" s="2">
         <v>76</v>
@@ -3656,7 +3643,7 @@
         <v>76</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>77</v>
@@ -3671,24 +3658,24 @@
         <v>76</v>
       </c>
       <c r="AK16" t="s" s="2">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="AM16" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AN16" t="s" s="2">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3711,16 +3698,16 @@
         <v>88</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
@@ -3770,39 +3757,39 @@
         <v>76</v>
       </c>
       <c r="AF17" t="s" s="2">
+        <v>196</v>
+      </c>
+      <c r="AG17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH17" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK17" t="s" s="2">
         <v>201</v>
       </c>
-      <c r="AG17" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH17" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI17" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ17" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK17" t="s" s="2">
-        <v>206</v>
-      </c>
       <c r="AL17" t="s" s="2">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="AM17" t="s" s="2">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="AN17" t="s" s="2">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3825,16 +3812,16 @@
         <v>88</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -3884,39 +3871,39 @@
         <v>76</v>
       </c>
       <c r="AF18" t="s" s="2">
+        <v>205</v>
+      </c>
+      <c r="AG18" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH18" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK18" t="s" s="2">
         <v>210</v>
       </c>
-      <c r="AG18" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH18" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI18" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ18" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK18" t="s" s="2">
-        <v>215</v>
-      </c>
       <c r="AL18" t="s" s="2">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="AM18" t="s" s="2">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="AN18" t="s" s="2">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3939,16 +3926,16 @@
         <v>88</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
@@ -3998,39 +3985,39 @@
         <v>76</v>
       </c>
       <c r="AF19" t="s" s="2">
+        <v>214</v>
+      </c>
+      <c r="AG19" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AH19" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK19" t="s" s="2">
         <v>219</v>
       </c>
-      <c r="AG19" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AH19" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI19" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ19" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK19" t="s" s="2">
-        <v>224</v>
-      </c>
       <c r="AL19" t="s" s="2">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="AM19" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AN19" t="s" s="2">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -4053,16 +4040,16 @@
         <v>88</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -4112,7 +4099,7 @@
         <v>76</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>77</v>
@@ -4127,24 +4114,24 @@
         <v>76</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="AN20" t="s" s="2">
-        <v>234</v>
+        <v>229</v>
       </c>
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -4167,16 +4154,16 @@
         <v>88</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
@@ -4226,39 +4213,39 @@
         <v>76</v>
       </c>
       <c r="AF21" t="s" s="2">
+        <v>230</v>
+      </c>
+      <c r="AG21" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH21" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK21" t="s" s="2">
         <v>235</v>
       </c>
-      <c r="AG21" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH21" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI21" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ21" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK21" t="s" s="2">
-        <v>240</v>
-      </c>
       <c r="AL21" t="s" s="2">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="AM21" t="s" s="2">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="AN21" t="s" s="2">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4281,13 +4268,13 @@
         <v>88</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="N22" t="s" s="2">
         <v>173</v>
@@ -4340,7 +4327,7 @@
         <v>76</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>77</v>
@@ -4355,7 +4342,7 @@
         <v>76</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="AL22" t="s" s="2">
         <v>76</v>
@@ -4369,10 +4356,10 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -4395,16 +4382,16 @@
         <v>88</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -4454,7 +4441,7 @@
         <v>76</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>77</v>
@@ -4466,10 +4453,10 @@
         <v>76</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="AL23" t="s" s="2">
         <v>76</v>
@@ -4483,10 +4470,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4509,13 +4496,13 @@
         <v>76</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -4566,7 +4553,7 @@
         <v>76</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>77</v>
@@ -4581,7 +4568,7 @@
         <v>76</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL24" t="s" s="2">
         <v>76</v>
@@ -4595,10 +4582,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4627,7 +4614,7 @@
         <v>134</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="N25" t="s" s="2">
         <v>136</v>
@@ -4680,7 +4667,7 @@
         <v>76</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>77</v>
@@ -4695,7 +4682,7 @@
         <v>76</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL25" t="s" s="2">
         <v>76</v>
@@ -4709,14 +4696,14 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
@@ -4741,7 +4728,7 @@
         <v>139</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="N26" t="s" s="2">
         <v>136</v>
@@ -4794,7 +4781,7 @@
         <v>76</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>77</v>
@@ -4823,10 +4810,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4852,13 +4839,13 @@
         <v>106</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
@@ -4887,10 +4874,10 @@
         <v>163</v>
       </c>
       <c r="Y27" t="s" s="2">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="Z27" t="s" s="2">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="AA27" t="s" s="2">
         <v>76</v>
@@ -4908,7 +4895,7 @@
         <v>76</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>87</v>
@@ -4923,7 +4910,7 @@
         <v>76</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="AL27" t="s" s="2">
         <v>76</v>
@@ -4932,15 +4919,15 @@
         <v>76</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4963,13 +4950,13 @@
         <v>88</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -5020,39 +5007,39 @@
         <v>76</v>
       </c>
       <c r="AF28" t="s" s="2">
+        <v>272</v>
+      </c>
+      <c r="AG28" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AH28" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK28" t="s" s="2">
+        <v>276</v>
+      </c>
+      <c r="AL28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AM28" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AN28" t="s" s="2">
         <v>277</v>
-      </c>
-      <c r="AG28" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AH28" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI28" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ28" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK28" t="s" s="2">
-        <v>281</v>
-      </c>
-      <c r="AL28" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AM28" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AN28" t="s" s="2">
-        <v>282</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -5075,19 +5062,19 @@
         <v>88</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="O29" t="s" s="2">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>76</v>
@@ -5136,39 +5123,39 @@
         <v>76</v>
       </c>
       <c r="AF29" t="s" s="2">
+        <v>278</v>
+      </c>
+      <c r="AG29" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH29" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ29" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK29" t="s" s="2">
         <v>283</v>
       </c>
-      <c r="AG29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH29" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI29" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ29" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK29" t="s" s="2">
-        <v>288</v>
-      </c>
       <c r="AL29" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>290</v>
+        <v>285</v>
       </c>
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5194,16 +5181,16 @@
         <v>179</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="O30" t="s" s="2">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="P30" t="s" s="2">
         <v>76</v>
@@ -5231,10 +5218,10 @@
         <v>110</v>
       </c>
       <c r="Y30" t="s" s="2">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="Z30" t="s" s="2">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="AA30" t="s" s="2">
         <v>76</v>
@@ -5252,7 +5239,7 @@
         <v>76</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>77</v>
@@ -5267,24 +5254,24 @@
         <v>76</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="AL30" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>300</v>
+        <v>295</v>
       </c>
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -5307,13 +5294,13 @@
         <v>88</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -5364,7 +5351,7 @@
         <v>76</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>87</v>
@@ -5376,10 +5363,10 @@
         <v>76</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>76</v>
@@ -5393,10 +5380,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5419,13 +5406,13 @@
         <v>76</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -5476,7 +5463,7 @@
         <v>76</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>77</v>
@@ -5491,7 +5478,7 @@
         <v>76</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL32" t="s" s="2">
         <v>76</v>
@@ -5505,10 +5492,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5537,7 +5524,7 @@
         <v>134</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="N33" t="s" s="2">
         <v>136</v>
@@ -5590,7 +5577,7 @@
         <v>76</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>77</v>
@@ -5605,7 +5592,7 @@
         <v>76</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>76</v>
@@ -5619,14 +5606,14 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
@@ -5651,7 +5638,7 @@
         <v>139</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="N34" t="s" s="2">
         <v>136</v>
@@ -5704,7 +5691,7 @@
         <v>76</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>77</v>
@@ -5733,10 +5720,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5759,13 +5746,13 @@
         <v>88</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -5816,39 +5803,39 @@
         <v>76</v>
       </c>
       <c r="AF35" t="s" s="2">
+        <v>303</v>
+      </c>
+      <c r="AG35" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AH35" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI35" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ35" t="s" s="2">
+        <v>307</v>
+      </c>
+      <c r="AK35" t="s" s="2">
+        <v>299</v>
+      </c>
+      <c r="AL35" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AM35" t="s" s="2">
         <v>308</v>
       </c>
-      <c r="AG35" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AH35" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ35" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="AK35" t="s" s="2">
-        <v>304</v>
-      </c>
-      <c r="AL35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AM35" t="s" s="2">
-        <v>313</v>
-      </c>
       <c r="AN35" t="s" s="2">
-        <v>314</v>
+        <v>309</v>
       </c>
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5871,13 +5858,13 @@
         <v>76</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5928,7 +5915,7 @@
         <v>76</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>77</v>
@@ -5943,7 +5930,7 @@
         <v>76</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>76</v>
@@ -5957,10 +5944,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5989,7 +5976,7 @@
         <v>134</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="N37" t="s" s="2">
         <v>136</v>
@@ -6030,19 +6017,19 @@
         <v>76</v>
       </c>
       <c r="AB37" t="s" s="2">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="AC37" t="s" s="2">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="AD37" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE37" t="s" s="2">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>77</v>
@@ -6057,7 +6044,7 @@
         <v>76</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>76</v>
@@ -6071,10 +6058,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6100,14 +6087,14 @@
         <v>106</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" t="s" s="2">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="P38" t="s" s="2">
         <v>76</v>
@@ -6120,7 +6107,7 @@
         <v>76</v>
       </c>
       <c r="T38" t="s" s="2">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="U38" t="s" s="2">
         <v>76</v>
@@ -6135,10 +6122,10 @@
         <v>163</v>
       </c>
       <c r="Y38" t="s" s="2">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="Z38" t="s" s="2">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="AA38" t="s" s="2">
         <v>76</v>
@@ -6156,7 +6143,7 @@
         <v>76</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>77</v>
@@ -6171,13 +6158,13 @@
         <v>76</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="AN38" t="s" s="2">
         <v>76</v>
@@ -6185,10 +6172,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6214,14 +6201,14 @@
         <v>106</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" t="s" s="2">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="P39" t="s" s="2">
         <v>76</v>
@@ -6234,7 +6221,7 @@
         <v>76</v>
       </c>
       <c r="T39" t="s" s="2">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="U39" t="s" s="2">
         <v>76</v>
@@ -6270,7 +6257,7 @@
         <v>76</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>77</v>
@@ -6285,7 +6272,7 @@
         <v>76</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>76</v>
@@ -6299,10 +6286,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6325,19 +6312,19 @@
         <v>76</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="N40" t="s" s="2">
         <v>173</v>
       </c>
       <c r="O40" t="s" s="2">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="P40" t="s" s="2">
         <v>76</v>
@@ -6386,7 +6373,7 @@
         <v>76</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>77</v>
@@ -6401,13 +6388,13 @@
         <v>76</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="AL40" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="AN40" t="s" s="2">
         <v>76</v>
@@ -6415,10 +6402,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6444,16 +6431,16 @@
         <v>100</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="N41" t="s" s="2">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="O41" t="s" s="2">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="P41" t="s" s="2">
         <v>76</v>
@@ -6466,7 +6453,7 @@
         <v>76</v>
       </c>
       <c r="T41" t="s" s="2">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="U41" t="s" s="2">
         <v>76</v>
@@ -6502,7 +6489,7 @@
         <v>76</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>77</v>
@@ -6517,13 +6504,13 @@
         <v>76</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="AL41" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="AN41" t="s" s="2">
         <v>76</v>
@@ -6531,10 +6518,10 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6557,19 +6544,19 @@
         <v>88</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="O42" t="s" s="2">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="P42" t="s" s="2">
         <v>76</v>
@@ -6618,7 +6605,7 @@
         <v>76</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>77</v>
@@ -6633,7 +6620,7 @@
         <v>76</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="AL42" t="s" s="2">
         <v>76</v>
@@ -6647,10 +6634,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6673,19 +6660,19 @@
         <v>88</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="N43" t="s" s="2">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="O43" t="s" s="2">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="P43" t="s" s="2">
         <v>76</v>
@@ -6734,7 +6721,7 @@
         <v>76</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>77</v>
@@ -6749,7 +6736,7 @@
         <v>76</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="AL43" t="s" s="2">
         <v>76</v>
@@ -6763,10 +6750,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6789,17 +6776,17 @@
         <v>88</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" t="s" s="2">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="P44" t="s" s="2">
         <v>76</v>
@@ -6812,7 +6799,7 @@
         <v>76</v>
       </c>
       <c r="T44" t="s" s="2">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="U44" t="s" s="2">
         <v>76</v>
@@ -6848,7 +6835,7 @@
         <v>76</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>77</v>
@@ -6863,7 +6850,7 @@
         <v>76</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>76</v>
@@ -6877,10 +6864,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6903,19 +6890,19 @@
         <v>88</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="N45" t="s" s="2">
         <v>173</v>
       </c>
       <c r="O45" t="s" s="2">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="P45" t="s" s="2">
         <v>76</v>
@@ -6964,7 +6951,7 @@
         <v>76</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>77</v>
@@ -6979,7 +6966,7 @@
         <v>76</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>76</v>
@@ -6993,10 +6980,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7019,16 +7006,16 @@
         <v>88</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -7054,11 +7041,11 @@
         <v>76</v>
       </c>
       <c r="X46" t="s" s="2">
-        <v>183</v>
+        <v>381</v>
       </c>
       <c r="Y46" s="2"/>
       <c r="Z46" t="s" s="2">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="AA46" t="s" s="2">
         <v>76</v>
@@ -7076,7 +7063,7 @@
         <v>76</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>77</v>
@@ -7091,7 +7078,7 @@
         <v>76</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="AL46" t="s" s="2">
         <v>76</v>
@@ -7100,15 +7087,15 @@
         <v>76</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>387</v>
+        <v>383</v>
       </c>
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7131,16 +7118,16 @@
         <v>88</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -7190,22 +7177,22 @@
         <v>76</v>
       </c>
       <c r="AF47" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="AG47" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH47" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI47" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ47" t="s" s="2">
+        <v>249</v>
+      </c>
+      <c r="AK47" t="s" s="2">
         <v>388</v>
-      </c>
-      <c r="AG47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH47" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI47" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ47" t="s" s="2">
-        <v>254</v>
-      </c>
-      <c r="AK47" t="s" s="2">
-        <v>392</v>
       </c>
       <c r="AL47" t="s" s="2">
         <v>76</v>
@@ -7219,10 +7206,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7245,13 +7232,13 @@
         <v>76</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -7302,7 +7289,7 @@
         <v>76</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>77</v>
@@ -7317,7 +7304,7 @@
         <v>76</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL48" t="s" s="2">
         <v>76</v>
@@ -7331,10 +7318,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7363,7 +7350,7 @@
         <v>134</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="N49" t="s" s="2">
         <v>136</v>
@@ -7416,7 +7403,7 @@
         <v>76</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>77</v>
@@ -7431,7 +7418,7 @@
         <v>76</v>
       </c>
       <c r="AK49" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL49" t="s" s="2">
         <v>76</v>
@@ -7445,14 +7432,14 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
@@ -7477,7 +7464,7 @@
         <v>139</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="N50" t="s" s="2">
         <v>136</v>
@@ -7530,7 +7517,7 @@
         <v>76</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>77</v>
@@ -7559,10 +7546,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7585,16 +7572,16 @@
         <v>88</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="N51" t="s" s="2">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
@@ -7644,7 +7631,7 @@
         <v>76</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>77</v>
@@ -7659,10 +7646,10 @@
         <v>76</v>
       </c>
       <c r="AK51" t="s" s="2">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="AL51" t="s" s="2">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="AM51" t="s" s="2">
         <v>76</v>
@@ -7673,10 +7660,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7702,13 +7689,13 @@
         <v>179</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
@@ -7734,13 +7721,13 @@
         <v>76</v>
       </c>
       <c r="X52" t="s" s="2">
-        <v>196</v>
+        <v>403</v>
       </c>
       <c r="Y52" t="s" s="2">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="Z52" t="s" s="2">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="AA52" t="s" s="2">
         <v>76</v>
@@ -7758,7 +7745,7 @@
         <v>76</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>77</v>
@@ -7773,7 +7760,7 @@
         <v>76</v>
       </c>
       <c r="AK52" t="s" s="2">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="AL52" t="s" s="2">
         <v>76</v>
@@ -7782,15 +7769,15 @@
         <v>76</v>
       </c>
       <c r="AN52" t="s" s="2">
-        <v>410</v>
+        <v>407</v>
       </c>
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7813,13 +7800,13 @@
         <v>88</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
@@ -7870,7 +7857,7 @@
         <v>76</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>77</v>
@@ -7885,7 +7872,7 @@
         <v>76</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="AL53" t="s" s="2">
         <v>76</v>
@@ -7894,15 +7881,15 @@
         <v>76</v>
       </c>
       <c r="AN53" t="s" s="2">
-        <v>416</v>
+        <v>413</v>
       </c>
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -7925,13 +7912,13 @@
         <v>76</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -7982,7 +7969,7 @@
         <v>76</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>77</v>
@@ -7997,7 +7984,7 @@
         <v>76</v>
       </c>
       <c r="AK54" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL54" t="s" s="2">
         <v>76</v>
@@ -8011,10 +7998,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8043,7 +8030,7 @@
         <v>134</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="N55" t="s" s="2">
         <v>136</v>
@@ -8084,19 +8071,19 @@
         <v>76</v>
       </c>
       <c r="AB55" t="s" s="2">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="AC55" t="s" s="2">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="AD55" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE55" t="s" s="2">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>77</v>
@@ -8111,7 +8098,7 @@
         <v>76</v>
       </c>
       <c r="AK55" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL55" t="s" s="2">
         <v>76</v>
@@ -8125,10 +8112,10 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8151,16 +8138,16 @@
         <v>88</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="N56" t="s" s="2">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="O56" s="2"/>
       <c r="P56" t="s" s="2">
@@ -8210,28 +8197,28 @@
         <v>76</v>
       </c>
       <c r="AF56" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="AG56" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH56" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI56" t="s" s="2">
+        <v>421</v>
+      </c>
+      <c r="AJ56" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK56" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="AL56" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AM56" t="s" s="2">
         <v>423</v>
-      </c>
-      <c r="AG56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH56" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI56" t="s" s="2">
-        <v>424</v>
-      </c>
-      <c r="AJ56" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK56" t="s" s="2">
-        <v>425</v>
-      </c>
-      <c r="AL56" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AM56" t="s" s="2">
-        <v>426</v>
       </c>
       <c r="AN56" t="s" s="2">
         <v>76</v>
@@ -8239,10 +8226,10 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8265,89 +8252,89 @@
         <v>88</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="N57" t="s" s="2">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q57" t="s" s="2">
+        <v>428</v>
+      </c>
+      <c r="R57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF57" t="s" s="2">
+        <v>429</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>421</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK57" t="s" s="2">
+        <v>430</v>
+      </c>
+      <c r="AL57" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AM57" t="s" s="2">
         <v>431</v>
-      </c>
-      <c r="R57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="S57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="T57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="U57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="V57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="W57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="X57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Z57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AA57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AB57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AC57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AD57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AE57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AF57" t="s" s="2">
-        <v>432</v>
-      </c>
-      <c r="AG57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH57" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI57" t="s" s="2">
-        <v>424</v>
-      </c>
-      <c r="AJ57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK57" t="s" s="2">
-        <v>433</v>
-      </c>
-      <c r="AL57" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AM57" t="s" s="2">
-        <v>434</v>
       </c>
       <c r="AN57" t="s" s="2">
         <v>76</v>
@@ -8355,10 +8342,10 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8384,10 +8371,10 @@
         <v>179</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -8414,63 +8401,63 @@
         <v>76</v>
       </c>
       <c r="X58" t="s" s="2">
-        <v>196</v>
+        <v>403</v>
       </c>
       <c r="Y58" t="s" s="2">
+        <v>435</v>
+      </c>
+      <c r="Z58" t="s" s="2">
+        <v>436</v>
+      </c>
+      <c r="AA58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF58" t="s" s="2">
+        <v>432</v>
+      </c>
+      <c r="AG58" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH58" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK58" t="s" s="2">
+        <v>437</v>
+      </c>
+      <c r="AL58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AM58" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AN58" t="s" s="2">
         <v>438</v>
-      </c>
-      <c r="Z58" t="s" s="2">
-        <v>439</v>
-      </c>
-      <c r="AA58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AB58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AC58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AD58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AE58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AF58" t="s" s="2">
-        <v>435</v>
-      </c>
-      <c r="AG58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH58" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK58" t="s" s="2">
-        <v>440</v>
-      </c>
-      <c r="AL58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AM58" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AN58" t="s" s="2">
-        <v>441</v>
       </c>
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8496,16 +8483,16 @@
         <v>179</v>
       </c>
       <c r="L59" t="s" s="2">
+        <v>440</v>
+      </c>
+      <c r="M59" t="s" s="2">
+        <v>441</v>
+      </c>
+      <c r="N59" t="s" s="2">
+        <v>442</v>
+      </c>
+      <c r="O59" t="s" s="2">
         <v>443</v>
-      </c>
-      <c r="M59" t="s" s="2">
-        <v>444</v>
-      </c>
-      <c r="N59" t="s" s="2">
-        <v>445</v>
-      </c>
-      <c r="O59" t="s" s="2">
-        <v>446</v>
       </c>
       <c r="P59" t="s" s="2">
         <v>76</v>
@@ -8530,13 +8517,13 @@
         <v>76</v>
       </c>
       <c r="X59" t="s" s="2">
-        <v>196</v>
+        <v>403</v>
       </c>
       <c r="Y59" t="s" s="2">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="Z59" t="s" s="2">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="AA59" t="s" s="2">
         <v>76</v>
@@ -8554,7 +8541,7 @@
         <v>76</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>77</v>
@@ -8569,7 +8556,7 @@
         <v>76</v>
       </c>
       <c r="AK59" t="s" s="2">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="AL59" t="s" s="2">
         <v>76</v>
@@ -8578,15 +8565,15 @@
         <v>76</v>
       </c>
       <c r="AN59" t="s" s="2">
-        <v>449</v>
+        <v>446</v>
       </c>
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -8609,16 +8596,16 @@
         <v>88</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="N60" t="s" s="2">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
@@ -8668,7 +8655,7 @@
         <v>76</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>77</v>
@@ -8683,7 +8670,7 @@
         <v>76</v>
       </c>
       <c r="AK60" t="s" s="2">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="AL60" t="s" s="2">
         <v>76</v>
@@ -8692,15 +8679,15 @@
         <v>76</v>
       </c>
       <c r="AN60" t="s" s="2">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -8723,16 +8710,16 @@
         <v>88</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -8782,7 +8769,7 @@
         <v>76</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>77</v>
@@ -8794,10 +8781,10 @@
         <v>76</v>
       </c>
       <c r="AJ61" t="s" s="2">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="AK61" t="s" s="2">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="AL61" t="s" s="2">
         <v>76</v>
@@ -8806,15 +8793,15 @@
         <v>76</v>
       </c>
       <c r="AN61" t="s" s="2">
-        <v>460</v>
+        <v>457</v>
       </c>
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -8837,13 +8824,13 @@
         <v>76</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -8894,7 +8881,7 @@
         <v>76</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>77</v>
@@ -8909,7 +8896,7 @@
         <v>76</v>
       </c>
       <c r="AK62" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL62" t="s" s="2">
         <v>76</v>
@@ -8923,10 +8910,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -8955,7 +8942,7 @@
         <v>134</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="N63" t="s" s="2">
         <v>136</v>
@@ -9008,7 +8995,7 @@
         <v>76</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>77</v>
@@ -9023,7 +9010,7 @@
         <v>76</v>
       </c>
       <c r="AK63" t="s" s="2">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AL63" t="s" s="2">
         <v>76</v>
@@ -9037,14 +9024,14 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="E64" s="2"/>
       <c r="F64" t="s" s="2">
@@ -9069,7 +9056,7 @@
         <v>139</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="N64" t="s" s="2">
         <v>136</v>
@@ -9122,7 +9109,7 @@
         <v>76</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>77</v>
@@ -9151,10 +9138,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -9180,13 +9167,13 @@
         <v>143</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="N65" t="s" s="2">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="O65" s="2"/>
       <c r="P65" t="s" s="2">
@@ -9236,7 +9223,7 @@
         <v>76</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>77</v>
@@ -9251,7 +9238,7 @@
         <v>76</v>
       </c>
       <c r="AK65" t="s" s="2">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="AL65" t="s" s="2">
         <v>76</v>
@@ -9265,10 +9252,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -9291,16 +9278,16 @@
         <v>88</v>
       </c>
       <c r="K66" t="s" s="2">
+        <v>467</v>
+      </c>
+      <c r="L66" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="M66" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="N66" t="s" s="2">
         <v>470</v>
-      </c>
-      <c r="L66" t="s" s="2">
-        <v>471</v>
-      </c>
-      <c r="M66" t="s" s="2">
-        <v>472</v>
-      </c>
-      <c r="N66" t="s" s="2">
-        <v>473</v>
       </c>
       <c r="O66" s="2"/>
       <c r="P66" t="s" s="2">
@@ -9350,7 +9337,7 @@
         <v>76</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>77</v>
@@ -9365,7 +9352,7 @@
         <v>76</v>
       </c>
       <c r="AK66" t="s" s="2">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="AL66" t="s" s="2">
         <v>76</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@819fdee1bbf5a99cd6c93615bda59c9ef3b4a558 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-DocumentReference.xlsx
+++ b/StructureDefinition-DocumentReference.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-11-25T09:42:11+00:00</t>
+    <t>2024-11-25T11:02:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Verwijzingen naar documenten</t>
+    <t>Verwijzingen naar document</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>